<commit_message>
Versión final 1.0.0 — Limpieza y documentación para entrega
</commit_message>
<xml_diff>
--- a/estudiantes_validos.xlsx
+++ b/estudiantes_validos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\panch\Documents\Recuperacion2025\Uisek\Tesis\SISTEMAGESTIONPRACTICAS\CODIGO\ProyectoTesisBackend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB5525FA-E936-49ED-B285-178A1197EB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4D5CC8-B723-4C59-98E9-3F48B55ACD87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="69">
   <si>
     <t>cedula</t>
   </si>
@@ -57,14 +57,188 @@
     <t>Morales</t>
   </si>
   <si>
-    <t>diego@uisek.edu.ec</t>
+    <t>diego.morales@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0001</t>
+  </si>
+  <si>
+    <t>Ana</t>
+  </si>
+  <si>
+    <t>Castro</t>
+  </si>
+  <si>
+    <t>ana.castro@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0002</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Vega</t>
+  </si>
+  <si>
+    <t>luis.vega@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>Informática</t>
+  </si>
+  <si>
+    <t>2026-0003</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>Torres</t>
+  </si>
+  <si>
+    <t>maria.torres@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>Negocios Internacionales</t>
+  </si>
+  <si>
+    <t>2026-0004</t>
+  </si>
+  <si>
+    <t>Carlos</t>
+  </si>
+  <si>
+    <t>Lopez</t>
+  </si>
+  <si>
+    <t>carlos.lopez@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0005</t>
+  </si>
+  <si>
+    <t>Rojas</t>
+  </si>
+  <si>
+    <t>Administración de Empresas</t>
+  </si>
+  <si>
+    <t>Pedro</t>
+  </si>
+  <si>
+    <t>Ruiz</t>
+  </si>
+  <si>
+    <t>pedro.ruiz@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0007</t>
+  </si>
+  <si>
+    <t>Flores</t>
+  </si>
+  <si>
+    <t>laura.flores@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0008</t>
+  </si>
+  <si>
+    <t>Andres</t>
+  </si>
+  <si>
+    <t>Salazar</t>
+  </si>
+  <si>
+    <t>andres.salazar@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0009</t>
+  </si>
+  <si>
+    <t>Camila</t>
+  </si>
+  <si>
+    <t>Herrera</t>
+  </si>
+  <si>
+    <t>camila.herrera@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0010</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Jimenez</t>
+  </si>
+  <si>
+    <t>david.jimenez@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0011</t>
+  </si>
+  <si>
+    <t>Valentina</t>
+  </si>
+  <si>
+    <t>Ortiz</t>
+  </si>
+  <si>
+    <t>valentina.ortiz@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0012</t>
+  </si>
+  <si>
+    <t>Sebastian</t>
+  </si>
+  <si>
+    <t>Mendoza</t>
+  </si>
+  <si>
+    <t>sebastian.mendoza@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0013</t>
+  </si>
+  <si>
+    <t>Daniela</t>
+  </si>
+  <si>
+    <t>Ponce</t>
+  </si>
+  <si>
+    <t>daniela.ponce@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0014</t>
+  </si>
+  <si>
+    <t>Alejandro</t>
+  </si>
+  <si>
+    <t>Quintero</t>
+  </si>
+  <si>
+    <t>alejandro.quintero@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0015</t>
+  </si>
+  <si>
+    <t>ana.rojas@uisek.edu.ec</t>
+  </si>
+  <si>
+    <t>2026-0016</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,14 +258,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -118,20 +284,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -413,11 +571,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="2" max="2" width="19" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="5" max="5" width="24.42578125" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="32.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -443,31 +606,356 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1766666666</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2">
         <v>996666666</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
-      <c r="G2" s="4"/>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1777777777</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3">
+        <v>997777777</v>
+      </c>
+      <c r="F3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1788888888</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4">
+        <v>998888888</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1799999999</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5">
+        <v>999999999</v>
+      </c>
+      <c r="F5" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1711111111</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6">
+        <v>991111111</v>
+      </c>
+      <c r="F6" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>172244422</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7">
+        <v>992112222</v>
+      </c>
+      <c r="F7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1733333333</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E8">
+        <v>993333333</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>1744111144</v>
+      </c>
+      <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9">
+        <v>994444444</v>
+      </c>
+      <c r="F9" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>1755555555</v>
+      </c>
+      <c r="B10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10">
+        <v>995555555</v>
+      </c>
+      <c r="F10" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1700000000</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11">
+        <v>990000000</v>
+      </c>
+      <c r="F11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>1712345678</v>
+      </c>
+      <c r="B12" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12">
+        <v>981234567</v>
+      </c>
+      <c r="F12" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1723456789</v>
+      </c>
+      <c r="B13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13">
+        <v>982345678</v>
+      </c>
+      <c r="F13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>1734567890</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14">
+        <v>983456789</v>
+      </c>
+      <c r="F14" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>1745678901</v>
+      </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15">
+        <v>984567890</v>
+      </c>
+      <c r="F15" t="s">
+        <v>24</v>
+      </c>
+      <c r="G15" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>1756789012</v>
+      </c>
+      <c r="B16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16">
+        <v>985678901</v>
+      </c>
+      <c r="F16" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" t="s">
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="mailto:diego@uisek.edu.ec" xr:uid="{6D99A252-0974-45F2-B4C7-51A3D86BA29E}"/>
+    <hyperlink ref="D7" r:id="rId1" xr:uid="{49935768-8492-452B-B3D6-D7D641E98BFB}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>